<commit_message>
feat: implementar configuracion de comprobantes, mejoras en ventas y ajustes de importacion de productos
</commit_message>
<xml_diff>
--- a/productos_import_masivo_actualizado.xlsx
+++ b/productos_import_masivo_actualizado.xlsx
@@ -9,8 +9,8 @@
 <cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <dc:creator>Codex</dc:creator>
   <cp:lastModifiedBy>Codex</cp:lastModifiedBy>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-02-27T18:21:58Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-02-27T18:21:58Z</dcterms:modified>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-03-03T23:16:51Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-03T23:16:51Z</dcterms:modified>
 </cp:coreProperties>
 </file>
 
@@ -68,32 +68,32 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>codigoExterno</t>
+          <t>categoriaNombre</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>categoriaNombre</t>
+          <t>colorNombre</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>colorNombre</t>
+          <t>colorHex</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>colorHex</t>
+          <t>tallaNombre</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>tallaNombre</t>
+          <t>precio</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>precio</t>
+          <t>precioOferta</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
@@ -125,31 +125,29 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>EXT-CHO-200-NEG-S</t>
+          <t>Chompas</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Chompas</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Negro</t>
+          <t>#111111</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>#111111</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>S</t>
         </is>
       </c>
+      <c r="H2">
+        <v>149</v>
+      </c>
       <c r="I2">
-        <v>149</v>
+        <v>129</v>
       </c>
       <c r="J2">
         <v>9</v>
@@ -178,31 +176,29 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>EXT-CHO-200-NEG-M</t>
+          <t>Chompas</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Chompas</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Negro</t>
+          <t>#111111</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>#111111</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
           <t>M</t>
         </is>
       </c>
+      <c r="H3">
+        <v>149</v>
+      </c>
       <c r="I3">
-        <v>149</v>
+        <v>129</v>
       </c>
       <c r="J3">
         <v>8</v>
@@ -231,31 +227,31 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>EXT-CHO-200-BEI-M</t>
+          <t>Chompas</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Chompas</t>
+          <t>Beige</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Beige</t>
+          <t>#D6C6A5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>#D6C6A5</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I4">
+      <c r="H4">
         <v>152</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J4">
         <v>7</v>
@@ -284,31 +280,29 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>EXT-VES-310-AZU-M</t>
+          <t>Vestidos</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Vestidos</t>
+          <t>Azul Cobalto</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Azul Cobalto</t>
+          <t>#0047AB</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>#0047AB</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
           <t>M</t>
         </is>
       </c>
+      <c r="H5">
+        <v>179.9</v>
+      </c>
       <c r="I5">
-        <v>179.9</v>
+        <v>169.9</v>
       </c>
       <c r="J5">
         <v>6</v>
@@ -337,31 +331,29 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EXT-VES-310-AZU-L</t>
+          <t>Vestidos</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Vestidos</t>
+          <t>Azul Cobalto</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Azul Cobalto</t>
+          <t>#0047AB</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>#0047AB</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
           <t>L</t>
         </is>
       </c>
+      <c r="H6">
+        <v>179.9</v>
+      </c>
       <c r="I6">
-        <v>179.9</v>
+        <v>169.9</v>
       </c>
       <c r="J6">
         <v>5</v>
@@ -390,31 +382,31 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EXT-VES-310-ROS-M</t>
+          <t>Vestidos</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Vestidos</t>
+          <t>Rosa Palo</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Rosa Palo</t>
+          <t>#E8B4BC</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>#E8B4BC</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I7">
+      <c r="H7">
         <v>182.5</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J7">
         <v>4</v>
@@ -443,31 +435,29 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EXT-SHU-050-BLA-36</t>
+          <t>Calzado</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Calzado</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Blanco</t>
+          <t>#FFFFFF</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>#FFFFFF</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
           <t>36</t>
         </is>
       </c>
+      <c r="H8">
+        <v>129</v>
+      </c>
       <c r="I8">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="J8">
         <v>12</v>
@@ -496,31 +486,29 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EXT-SHU-050-BLA-37</t>
+          <t>Calzado</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Calzado</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Blanco</t>
+          <t>#FFFFFF</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>#FFFFFF</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
           <t>37</t>
         </is>
       </c>
+      <c r="H9">
+        <v>129</v>
+      </c>
       <c r="I9">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="J9">
         <v>11</v>
@@ -549,31 +537,31 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>EXT-SHU-050-GRI-37</t>
+          <t>Calzado</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Calzado</t>
+          <t>Gris Nube</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Gris Nube</t>
+          <t/>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
           <t>37</t>
         </is>
       </c>
-      <c r="I10">
+      <c r="H10">
         <v>131</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J10">
         <v>10</v>
@@ -602,31 +590,29 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EXT-POL-777-LIL-M</t>
+          <t>Polos</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Polos</t>
+          <t>Lila Vibrante</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Lila Vibrante</t>
+          <t>#B57EDC</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>#B57EDC</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
           <t>M</t>
         </is>
       </c>
+      <c r="H11">
+        <v>69.9</v>
+      </c>
       <c r="I11">
-        <v>69.9</v>
+        <v>59.9</v>
       </c>
       <c r="J11">
         <v>20</v>
@@ -655,31 +641,29 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EXT-POL-777-LIL-L</t>
+          <t>Polos</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Polos</t>
+          <t>Lila Vibrante</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Lila Vibrante</t>
+          <t>#B57EDC</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>#B57EDC</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
           <t>L</t>
         </is>
       </c>
+      <c r="H12">
+        <v>69.9</v>
+      </c>
       <c r="I12">
-        <v>69.9</v>
+        <v>59.9</v>
       </c>
       <c r="J12">
         <v>18</v>
@@ -708,31 +692,31 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t/>
+          <t>Polos</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Polos</t>
+          <t>Verde Lima</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Verde Lima</t>
+          <t>#32CD32</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>#32CD32</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
           <t>M</t>
         </is>
       </c>
-      <c r="I13">
+      <c r="H13">
         <v>71.5</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J13">
         <v>16</v>

</xml_diff>